<commit_message>
AR eval: Zainab ERP harvest (13 probes, data-presence PASSED, tool surface discovered), entities.json rebuilt, user query set enriched+labeled (56 rows, 54 ANSWER/2 CLARIFY)
</commit_message>
<xml_diff>
--- a/accounts/ar-agent/queries.xlsx
+++ b/accounts/ar-agent/queries.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,24 +450,24 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Position - Outstanding Snapshot</t>
+          <t>WhatsApp vs ERP Reconciliation</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>What is our total outstanding right now?</t>
+          <t>Which customers said payment is done on WhatsApp but it is still outstanding in ERP?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>position snapshot; latest date if omitted</t>
+          <t>core; reported claims vs ledger</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -479,17 +479,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>How much of our outstanding is overdue vs not yet due?</t>
+          <t>Which payments were claimed on WhatsApp but I can't find in ERP?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>position buckets</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -501,17 +501,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Show me the ageing breakup of what customers owe.</t>
+          <t>Check the payment claims in WhatsApp against the ERP receipts.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>b_1_30..b_90+ buckets</t>
+          <t>hedge: both sides presented, no auto-reconcile claim</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -523,17 +523,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Which customer has the highest outstanding?</t>
+          <t>Who says they paid, but we haven't received it in our books?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>position sorted desc</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -545,17 +545,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Who are our top 5 by outstanding?</t>
+          <t>Find payment claims with no matching ERP receipt — like KRISHNA COATED FABRICS, POPULAR MATTRESS &amp; CLOTH STORE, TRENDS FURNISHING.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>upper management, plain language</t>
+          <t>anchored: the 10-claim ₹7,41,130 set</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -567,17 +567,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Is this outstanding figure up to date?</t>
+          <t>Which WhatsApp payments are still unreconciled?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>stale snapshot -&gt; 'latest list is from &lt;date&gt;' (never the word stale)</t>
+          <t>[lenient] unreconciled = judgment</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -589,17 +589,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>What did our outstanding look like as of last month's snapshot?</t>
+          <t>Show me payments where the WhatsApp amount doesn't match the ERP amount.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>as_of param</t>
+          <t>[lenient] amount-compare judgment</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -611,17 +611,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Which customers have no outstanding at all?</t>
+          <t>Who paid partially in ERP even though they said full payment on WhatsApp?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>zero-balance list</t>
+          <t>[lenient] partial-vs-full judgment; chain get_receivables</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -633,17 +633,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Has our total outstanding changed much vs the previous snapshot?</t>
+          <t>Which customers shared a UTR on WhatsApp but there is no matching receipt in ERP?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>trend honesty: DSO/collections history unavailable by design</t>
+          <t>[lenient] UTR-matching judgment; chain get_receivables</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -653,48 +653,48 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Worklist - Priority &amp; Chase</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Any payment claims from WhatsApp that need verification?</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ar_payments_reported</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Who do we chase first today?</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>worklist rank is AUTHORITATIVE - never re-rank by opinion</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>TOOL:query_ar</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Payment Commitment Follow-up</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Show the top of the chase list with days past due.</t>
+          <t>Who promised to pay this week but still has an outstanding balance?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>chaseable_balance + days_past_due</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_promises</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -706,17 +706,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Which 5 customers should we prioritize for collection today?</t>
+          <t>Who said on WhatsApp they'll pay tomorrow?</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>upper management, plain language</t>
+          <t>chain search_threads</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_promises</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -728,17 +728,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Who is on hold right now and why?</t>
+          <t>Which promised payments are overdue now — like the ONCE &amp; AGAIN commitment?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>held rows have null rank; suppression_object links</t>
+          <t>anchored; [lenient] promise-overdue judgment; chain ar_position</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_promises</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -750,17 +750,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>What is our next best follow-up?</t>
+          <t>Show me customers whose committed payment date has passed.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>upper management, plain language</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_promises</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -772,17 +772,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Where does Om Enterprises Traders 421 sit on the chase list?</t>
+          <t>Who keeps promising payment but hasn't cleared the dues?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>real customer</t>
+          <t>[lenient] 'keeps' = repeated commitments; chain get_receivables</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_promises</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -794,17 +794,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Are any holds linked to an open dispute?</t>
+          <t>Which WhatsApp payment commitments are still pending in ERP?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>WhatsApp-groundable</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_promises</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -816,17 +816,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Which customers did we follow up repeatedly?</t>
+          <t>Who gave a payment date on WhatsApp but no payment has been posted in ERP yet?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>UNCONFIRMABLE by design (activity = last_inbound/outbound only) - expect honest limitation</t>
+          <t>chain ar_payments_reported</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_promises</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -838,17 +838,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Should we chase anyone today?</t>
+          <t>Show me customers who said payment is scheduled but ERP still shows outstanding.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>upper management, plain language</t>
+          <t>chain get_receivables</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_promises</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -860,24 +860,24 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>Objects - WhatsApp Signals</t>
+          <t>Invoice / Bill Level</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Are there new payment claims in the groups?</t>
+          <t>Which invoices were mentioned as paid on WhatsApp but are still open in ERP?</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>WhatsApp-groundable</t>
+          <t>chain list_invoices</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -889,17 +889,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Who committed to paying this week?</t>
+          <t>Bill 15293 was claimed as paid on WhatsApp (NEFT ₹880) — is it in ERP?</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>objects type=commitment</t>
+          <t>anchored: REAL mismatch — ERP says NOT FOUND (doc_number filter)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>list_invoices</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -911,17 +911,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Which customers acknowledged their dues in WhatsApp?</t>
+          <t>Which bills have payment claims but no receipt entry?</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>objects type=acknowledgement</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -933,17 +933,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Any disputes raised in the groups?</t>
+          <t>Show me the overdue bills where the customer has already promised payment — e.g. the 91-day worklist accounts.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>objects type=dispute</t>
+          <t>anchored: RICH DECOR/EMBELLISH 91d class; chain ar_promises; [lenient] overdue = position</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_worklist</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -955,17 +955,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Have any cheques been promised?</t>
+          <t>Which invoice payments are pending despite customer confirmation on WhatsApp?</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>objects type=cheque</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -977,17 +977,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Who asked for a ledger copy or document in the groups?</t>
+          <t>Find bills where the WhatsApp amount and the ERP receipt don't match.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>objects type=document_request; WA</t>
+          <t>[lenient] amount-compare judgment</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -999,17 +999,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Om Enterprises Traders 421 said the payment is done - does the data confirm it?</t>
+          <t>Which customers mentioned specific invoice numbers while discussing payment — like 15293 or the ₹880 NEFT claim?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>claim reported != bank-verified; unknown amount != zero</t>
+          <t>anchored: invoice-number mentions in chat</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1019,41 +1019,26 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>What did Sai Agencies &amp; Co 1051 commit to paying?</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>resolve then objects; WA</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>TOOL:resolve_ar_identity</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>UTR / Reference Matching</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Any claims with an expected payment date this week?</t>
+          <t>Check the UTRs shared on WhatsApp against the ERP receipts.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>expected_date filter; WA</t>
+          <t>hedge: both sides presented</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1065,17 +1050,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Which open claims are suppressing our chasing?</t>
+          <t>Which UTRs don't have a matching entry in ERP?</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>suppresses_chasing; WA</t>
+          <t>[lenient] matching judgment; chain get_receivables</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1087,17 +1072,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Is there a hold because of a dispute from Krishna Traders LLP 125?</t>
+          <t>Show me payment claims where the reference number matches an ERP receipt.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>real customer; resolve -&gt; objects -&gt; worklist hold</t>
+          <t>[lenient] matching judgment</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>TOOL:resolve_ar_identity</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1109,17 +1094,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Any recent payment claims from Radha Agencies Pvt Ltd 787?</t>
+          <t>Are there any duplicate payment claims in WhatsApp?</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>real customer (the 2nd Radha - ambiguity pair with LLP 552); WA</t>
+          <t>[lenient] dedupe judgment</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>TOOL:query_ar</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1129,26 +1114,41 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>Financials - Invoices &amp; Balances</t>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Find payments where the UTR exists in WhatsApp but the receipt is missing in ERP.</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>[lenient] matching judgment; chain get_receivables</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>search_threads</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Show me the current balance of Ganesh Wholesalers Pvt Ltd 955.</t>
+          <t>Which payment references are still unresolved?</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>customer_balances; real customer</t>
+          <t>[lenient] unresolved = judgment</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>TOOL:query_ar_financials</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1158,41 +1158,26 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Which invoices are still open for Krishna Traders LLP 125?</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>invoices dataset</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>TOOL:query_ar_financials</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>Credit Note Scenarios</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>What is the ledger balance of Sai Agencies &amp; Co 1051?</t>
+          <t>Who is waiting for a credit note before making payment?</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>customer_balances</t>
+          <t>[lenient] CN surface UNVERIFIED on Zainab — expect hedge</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>TOOL:query_ar_financials</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1204,17 +1189,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Show me the most recent open invoices.</t>
+          <t>Which payments are stuck because of pending credit notes?</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>invoices; app renders rows</t>
+          <t>[lenient] CN surface unverified</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>TOOL:query_ar_financials</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1226,17 +1211,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Invoiced vs paid totals for Durga Traders Traders 811?</t>
+          <t>Find customers who said they'll pay after a credit note adjustment.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>real customer</t>
+          <t>[lenient] CN surface unverified</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>TOOL:query_ar_financials</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1248,17 +1233,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>What is the outstanding summary for Jai Wholesalers &amp; Co 918?</t>
+          <t>How much is pending after the credit note mentioned on WhatsApp?</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>resolve -&gt; financials</t>
+          <t>[lenient] CN surface unverified; chain get_receivables</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>TOOL:resolve_ar_identity</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1270,17 +1255,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Show me invoice 12859 and its payment status.</t>
+          <t>Which credit notes discussed in WhatsApp are still not reflected in ERP?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>REAL invoice from live discovery (Rs.900)</t>
+          <t>[lenient] CN surface unverified; chain get_receivables</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>TOOL:query_ar_financials</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1292,17 +1277,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Which customer's ledger moved the most this month?</t>
+          <t>Who asked for a credit note and still has an outstanding balance?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>upper management, plain language</t>
+          <t>[lenient] CN surface unverified; chain get_receivables</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>TOOL:query_ar_financials</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1314,17 +1299,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>What is the current balance of Lakshmi Distributors LLP 20?</t>
+          <t>Find cases where the customer says the credit note is pending but ERP already shows one.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>real customer</t>
+          <t>[lenient] both-sides CN compare</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>TOOL:query_ar_financials</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1336,24 +1321,24 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>Evidence</t>
+          <t>Repeated Follow-ups</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>What exactly did the customer say about the payment in the group?</t>
+          <t>Who have we chased multiple times but still haven't paid?</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>exact stored wording; authorize object first</t>
+          <t>chain search_threads</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>TOOL:get_ar_evidence</t>
+          <t>ar_worklist</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1365,17 +1350,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Show me the exact wording of Om Enterprises Traders 421's payment claim.</t>
+          <t>Which customers have repeated payment reminders in WhatsApp?</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>WhatsApp-groundable</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>TOOL:get_ar_evidence</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1387,17 +1372,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>What did Radha Agencies LLP 552 say about the cheque?</t>
+          <t>Show me the large outstanding customers with recent payment follow-ups — like Interworld Furnishings (₹7.24Cr).</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>real customer; evidence text + sender</t>
+          <t>anchored: Interworld ₹7.24Cr 91d</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>TOOL:get_ar_evidence</t>
+          <t>ar_worklist</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1409,17 +1394,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Can you show me the message where the commitment was made?</t>
+          <t>Who hasn't responded to our payment reminders?</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>WhatsApp-groundable</t>
+          <t>[lenient] response-status judgment</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>TOOL:get_ar_evidence</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1429,26 +1414,41 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="inlineStr">
-        <is>
-          <t>Paid Collections</t>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Which customers have acknowledged the dues but haven't paid?</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>acknowledged = commitment; chain get_receivables</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ar_promises</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>How much did we collect in total this month?</t>
+          <t>Find customers where payment follow-up repeats without any payment.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>workspace paid totals by payment date (status P)</t>
+          <t>[lenient] repeat+touch judgment; chain ar_payments_reported</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>TOOL:get_paid_collections</t>
+          <t>ar_worklist</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1458,41 +1458,26 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Compare this week's collections with last week's.</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>inclusive IST from/to</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>TOOL:get_paid_collections</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>Natural Accountant-style Queries</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Show me collections by payment date for this period.</t>
+          <t>What's the latest update on TRENDS FURNISHING's payment?</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>upper management, plain language</t>
+          <t>anchored (user's 'Palette' swapped — Palette unresolvable in Zainab balances; TRENDS FURNISHING has a real reported claim); chain search_threads</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>TOOL:get_paid_collections</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -1504,46 +1489,61 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Are collections improving month over month?</t>
+          <t>Did they actually pay this one?</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>period comparison; honest about scope - no customer breakdown</t>
+          <t>referent-less; tests the ask-back path</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>TOOL:get_paid_collections</t>
+          <t>ASK_BACK</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>CLARIFY</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="inlineStr">
-        <is>
-          <t>Conversation Snapshot</t>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>What did Interworld Furnishings say about their pending ₹7.24Cr in the chats?</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>anchored: Interworld ₹7.24Cr 91d; chain get_receivables</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>search_threads</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>What is the latest update in the HiraFoods-Om Enterprises Traders 421 group?</t>
+          <t>Has the payment for invoice 17346 been posted?</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>authorized 15-min window, NOT full history</t>
+          <t>anchored: real ERP invoice 17346 (₹27.73)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>TOOL:get_ar_conversation_snapshot</t>
+          <t>list_invoices</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -1555,17 +1555,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>What was the most recent message from Radha Agencies LLP 552?</t>
+          <t>They sent a UTR — can you check it? (the NEFT ₹880 claim against B NO 15293)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>WhatsApp-groundable</t>
+          <t>anchored: hiteshvthakkar ₹880 / B NO 15293 mismatch case; chain list_invoices</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>TOOL:get_ar_conversation_snapshot</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -1577,17 +1577,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>What was discussed around the Shree Retail Pvt Ltd 581 payment?</t>
+          <t>Check what KRISHNA COATED FABRICS said about their payment in the group and compare it with ERP.</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>real customer</t>
+          <t>anchored: real reported claim; chain ar_payments_reported</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>TOOL:get_ar_conversation_snapshot</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -1599,461 +1599,132 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Any activity on the Sri Retail &amp; Co 196 thread recently?</t>
+          <t>Why is this still showing outstanding when they said paid?</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>real customer</t>
+          <t>referent-less; tests the ask-back path</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>TOOL:get_ar_conversation_snapshot</t>
+          <t>ASK_BACK</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ANSWER</t>
+          <t>CLARIFY</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="inlineStr">
-        <is>
-          <t>Identity - Clarify &amp; Selection</t>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>How much is really pending for POPULAR MATTRESS &amp; CLOTH STORE after their WhatsApp-reported payment?</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>anchored: real reported claim; chain ar_payments_reported</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>get_receivables</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Tell me about Radha's outstanding.</t>
+          <t>For the customers who reported payments on WhatsApp, what are they waiting for from us?</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>TWO Radha accounts exist (LLP 552 + Pvt Ltd 787) - shortlist MUST be selected, even one row</t>
+          <t>[lenient] reason-extraction judgment</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>TOOL:resolve_ar_identity</t>
+          <t>search_threads</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>CLARIFY</t>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>What is the balance for Sai Agencies?</t>
+          <t>Who should I follow up with today based on the chats and ERP?</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>truncated name -&gt; shortlist</t>
+          <t>core — the worklist case</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>TOOL:resolve_ar_identity</t>
+          <t>ar_worklist</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>CLARIFY</t>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Who is Krishna Traders?</t>
+          <t>Give me the cases where WhatsApp and ERP don't agree.</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>fuzzy -&gt; shortlist</t>
+          <t>core — mismatch summary</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>TOOL:resolve_ar_identity</t>
+          <t>ar_payments_reported</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>CLARIFY</t>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>What does Om Enterprises owe us?</t>
+          <t>What's the current outstanding of Interworld Furnishings?</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>firm-only (no account number) -&gt; shortlist</t>
+          <t>identity-resolution gate: truncated-name vs ERP master 'Interworld Furnishings (I) Pvt. Ltd.' — expect resolve+answer, no fabricated amount</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>TOOL:resolve_ar_identity</t>
+          <t>search_customers_master</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>CLARIFY</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Check the dues for Shree Retail.</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>truncated -&gt; shortlist</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>TOOL:resolve_ar_identity</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>CLARIFY</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>What is Ganesh Wholesalers' position?</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>no number -&gt; shortlist</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>TOOL:resolve_ar_identity</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>CLARIFY</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Balance of Jai Wholesalers &amp; Co?</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>no number -&gt; shortlist</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>TOOL:resolve_ar_identity</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>CLARIFY</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="1" t="inlineStr">
-        <is>
-          <t>Plain-Language Upper Management</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Who owes us the most right now?</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>upper management, plain language</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>TOOL:query_ar</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Any big payments stuck?</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>upper management, plain language</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>TOOL:query_ar</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>What is the latest on the big payments?</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>objects + position; WA</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>TOOL:query_ar</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Where is most of our money stuck?</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>upper management, plain language</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>TOOL:query_ar</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Are our collections getting better?</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>upper management, plain language</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>TOOL:get_paid_collections</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Is anyone about to pay us this week?</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>expected_date commitments; WA</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>TOOL:query_ar</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>ANSWER</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="1" t="inlineStr">
-        <is>
-          <t>Unsupported - Read-Only Guard</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Verify in the bank that Om Enterprises Traders 421 paid us.</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>bank verification absent</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>NO_TOOL</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>REFUSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Forecast our collections for next quarter.</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>no forecasts (DSO/credit/cash)</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>NO_TOOL</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>REFUSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Mark Durga Traders Traders 811 as settled.</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>read-only - no writes ever</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>NO_TOOL</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>REFUSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Send a payment reminder to Sai Agencies &amp; Co 1051 on WhatsApp.</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>drafts only; sending is an authenticated UI action</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>NO_TOOL</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>REFUSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Show me which claims actually hit the bank account.</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>bank matching absent</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>NO_TOOL</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>REFUSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Confirm that Jai Wholesalers &amp; Co 918's cheque has cleared.</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>bank verification absent</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>NO_TOOL</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>REFUSE</t>
+          <t>ANSWER</t>
         </is>
       </c>
     </row>

</xml_diff>